<commit_message>
AI Job Hunter v7.0 Summary Email Release
</commit_message>
<xml_diff>
--- a/output/jobs.xlsx
+++ b/output/jobs.xlsx
@@ -464,7 +464,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5743507343?se=7OfVrRRu8RGnVKxb14Z7EQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EC3CE217025746C9731AE4A3FE3C1282A6011BCA</t>
+          <t>https://www.adzuna.in/land/ad/5743507343?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EC3CE217025746C9731AE4A3FE3C1282A6011BCA</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5730011191?se=7OfVrRRu8RGnVKxb14Z7EQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=32B1BBCA420C902A6F2C3E09000395AA8FE6A3F5</t>
+          <t>https://www.adzuna.in/land/ad/5730011191?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=32B1BBCA420C902A6F2C3E09000395AA8FE6A3F5</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279977?se=OEaUrhRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8140C4A63ACF7397C81D83F8A2E0D465705EC102</t>
+          <t>https://www.adzuna.in/land/ad/5769279977?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8140C4A63ACF7397C81D83F8A2E0D465705EC102</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742256993?se=7OfVrRRu8RGnVKxb14Z7EQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0C287C3961DC24298C835CB9417F8B09383F0052</t>
+          <t>https://www.adzuna.in/land/ad/5742256993?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0C287C3961DC24298C835CB9417F8B09383F0052</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763490875?se=7OfVrRRu8RGnVKxb14Z7EQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=F6580EC1E05F8A53AD05B2797EF5A9096F16DF5B</t>
+          <t>https://www.adzuna.in/land/ad/5763490875?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=F6580EC1E05F8A53AD05B2797EF5A9096F16DF5B</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763491420?se=OEaUrhRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3FBB99E390EDF9FEBCE53C278A62FE4664A860EC</t>
+          <t>https://www.adzuna.in/land/ad/5763491420?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3FBB99E390EDF9FEBCE53C278A62FE4664A860EC</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742256422?se=7OfVrRRu8RGnVKxb14Z7EQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=511A44A56B34F4F4124473FA10BE5E077D5B6C3D</t>
+          <t>https://www.adzuna.in/land/ad/5742256422?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=511A44A56B34F4F4124473FA10BE5E077D5B6C3D</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017767?se=ih_KsRRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1D57181F57C2D41E58572804A36F43C3D4AE9DD3</t>
+          <t>https://www.adzuna.in/land/ad/5768017767?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1D57181F57C2D41E58572804A36F43C3D4AE9DD3</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5751935354?se=oFtmrxRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F393812E08FBC954B1FB55EE1B56E2DFB50954C</t>
+          <t>https://www.adzuna.in/land/ad/5751935354?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F393812E08FBC954B1FB55EE1B56E2DFB50954C</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747040297?se=ih_KsRRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2E896599C4FAA7BFB268F9232FAAD133084B0921</t>
+          <t>https://www.adzuna.in/land/ad/5747040297?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2E896599C4FAA7BFB268F9232FAAD133084B0921</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753854888?se=ih_KsRRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=DCC65B6F5A7A335BD330AF1C5879E10E1A0DA2BF</t>
+          <t>https://www.adzuna.in/land/ad/5753854888?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=DCC65B6F5A7A335BD330AF1C5879E10E1A0DA2BF</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762127810?se=ih_KsRRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=55DA7A82770C696150F83F8133FACA98264C6E3F</t>
+          <t>https://www.adzuna.in/land/ad/5762127810?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=55DA7A82770C696150F83F8133FACA98264C6E3F</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5754995429?se=7OfVrRRu8RGnVKxb14Z7EQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=62BBB042D860B38D9BB38703AA92E62E26E7FEEF</t>
+          <t>https://www.adzuna.in/land/ad/5754995429?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=62BBB042D860B38D9BB38703AA92E62E26E7FEEF</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765773904?se=oFtmrxRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=13B225115728D3657DA50775D7912A9BA4ED36EB</t>
+          <t>https://www.adzuna.in/land/ad/5765773904?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=13B225115728D3657DA50775D7912A9BA4ED36EB</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765771294?se=7OfVrRRu8RGnVKxb14Z7EQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=66B0C0764A60AE7A967A48E96A0935EBE89724C7</t>
+          <t>https://www.adzuna.in/land/ad/5765771294?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=66B0C0764A60AE7A967A48E96A0935EBE89724C7</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5697518505?se=oFtmrxRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=9CEC78D19FCA0C7369A7A9F85A518FE1FD101D9B</t>
+          <t>https://www.adzuna.in/land/ad/5697518505?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=9CEC78D19FCA0C7369A7A9F85A518FE1FD101D9B</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753861658?se=ih_KsRRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2FEC94CE5CB423BFE26CF6D30B22638EDBB7E8F1</t>
+          <t>https://www.adzuna.in/land/ad/5753861658?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2FEC94CE5CB423BFE26CF6D30B22638EDBB7E8F1</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017975?se=OEaUrhRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=69D84AF1829A42AB98C8A52ADFD1EFCF7612FD49</t>
+          <t>https://www.adzuna.in/land/ad/5768017975?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=69D84AF1829A42AB98C8A52ADFD1EFCF7612FD49</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279314?se=OEaUrhRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D58B4AE61A5DFD6033A10582B36518DC793AE0F4</t>
+          <t>https://www.adzuna.in/land/ad/5769279314?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D58B4AE61A5DFD6033A10582B36518DC793AE0F4</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5718579853?se=ciozsBRu8RGl0MKcaJBBpg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EEB22977836DEAF81366ED7E9D416316985AA188</t>
+          <t>https://www.adzuna.in/land/ad/5718579853?se=Lq3IaR1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EEB22977836DEAF81366ED7E9D416316985AA188</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5771700968?se=ih_KsRRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=84E1AD6D342B54E01DADB5E011C6B186221EC596</t>
+          <t>https://www.adzuna.in/land/ad/5771700968?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=84E1AD6D342B54E01DADB5E011C6B186221EC596</t>
         </is>
       </c>
     </row>
@@ -989,7 +989,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753861185?se=oFtmrxRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=764A0D94268C270F0A11F41CD71DC452D8D024EE</t>
+          <t>https://www.adzuna.in/land/ad/5753861185?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=764A0D94268C270F0A11F41CD71DC452D8D024EE</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765775462?se=OEaUrhRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=37EF76F5E17E818F0447F6892E3D3033BCA9DEDB</t>
+          <t>https://www.adzuna.in/land/ad/5765775462?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=37EF76F5E17E818F0447F6892E3D3033BCA9DEDB</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747047144?se=ih_KsRRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=086536F916DBD1B18D3DC8ADC94A41EDB4152A26</t>
+          <t>https://www.adzuna.in/land/ad/5747047144?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=086536F916DBD1B18D3DC8ADC94A41EDB4152A26</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5751935153?se=ih_KsRRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=C4885E317E9A9D605051F18481BAC78ADCE69845</t>
+          <t>https://www.adzuna.in/land/ad/5751935153?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=C4885E317E9A9D605051F18481BAC78ADCE69845</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5750488988?se=nkMGsRRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D508B9EDA6796D7FEA984502C190316CE8C2A72B</t>
+          <t>https://www.adzuna.in/land/ad/5750488988?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D508B9EDA6796D7FEA984502C190316CE8C2A72B</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5724225887?se=oFtmrxRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=977640AFE7E1437C6FA9D94E36E92EE120B06CDA</t>
+          <t>https://www.adzuna.in/land/ad/5724225887?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=977640AFE7E1437C6FA9D94E36E92EE120B06CDA</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753195076?se=ciozsBRu8RGl0MKcaJBBpg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=923801176AE7A1C9773F36AF178EBD26D512CA14</t>
+          <t>https://www.adzuna.in/land/ad/5753195076?se=Lq3IaR1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=923801176AE7A1C9773F36AF178EBD26D512CA14</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763490809?se=oFtmrxRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2DE9C024149D8DBE2A1313F30D55C8D54F432F3D</t>
+          <t>https://www.adzuna.in/land/ad/5763490809?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2DE9C024149D8DBE2A1313F30D55C8D54F432F3D</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765772430?se=7OfVrRRu8RGnVKxb14Z7EQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=E53BCFC3CB04BBEBC29296EC5F4B42289617F051</t>
+          <t>https://www.adzuna.in/land/ad/5765772430?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=E53BCFC3CB04BBEBC29296EC5F4B42289617F051</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742257007?se=ciozsBRu8RGl0MKcaJBBpg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2D757BB48A163442E841856250996D40F30FC3E4</t>
+          <t>https://www.adzuna.in/land/ad/5742257007?se=Lq3IaR1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2D757BB48A163442E841856250996D40F30FC3E4</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745164418?se=ciozsBRu8RGl0MKcaJBBpg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3B0A759BCDB59AF4E25E85006C1AB1D0EB157057</t>
+          <t>https://www.adzuna.in/land/ad/5745164418?se=Lq3IaR1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3B0A759BCDB59AF4E25E85006C1AB1D0EB157057</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5771700899?se=OEaUrhRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EAC9690D3DACE0A8E1DB58475E6591E96A8C07DF</t>
+          <t>https://www.adzuna.in/land/ad/5771700899?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EAC9690D3DACE0A8E1DB58475E6591E96A8C07DF</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747049084?se=oFtmrxRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=125E41A1B9DDB57408262D54D83632341383D0EB</t>
+          <t>https://www.adzuna.in/land/ad/5747049084?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=125E41A1B9DDB57408262D54D83632341383D0EB</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5760048697?se=ih_KsRRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=70CA53C4D36C78E465CA1A70805E0139B2E3FFAB</t>
+          <t>https://www.adzuna.in/land/ad/5760048697?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=70CA53C4D36C78E465CA1A70805E0139B2E3FFAB</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5757284504?se=nkMGsRRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=FBC032DA8BAD5D3101B3CC9E54E5B69521B6E72A</t>
+          <t>https://www.adzuna.in/land/ad/5757284504?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=FBC032DA8BAD5D3101B3CC9E54E5B69521B6E72A</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763491377?se=OEaUrhRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4B3A4958BCF6866E580142C09980F0C770C32C7</t>
+          <t>https://www.adzuna.in/land/ad/5763491377?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4B3A4958BCF6866E580142C09980F0C770C32C7</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017288?se=7OfVrRRu8RGnVKxb14Z7EQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=83958946379D0B2DA69D00F6C975FEC5992724E7</t>
+          <t>https://www.adzuna.in/land/ad/5768017288?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=83958946379D0B2DA69D00F6C975FEC5992724E7</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753191970?se=oFtmrxRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6BDA6CC2A00FC003582875F486E3C68BB692E1A3</t>
+          <t>https://www.adzuna.in/land/ad/5753191970?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6BDA6CC2A00FC003582875F486E3C68BB692E1A3</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5750495104?se=ciozsBRu8RGl0MKcaJBBpg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=BEB267C4FE33B892711F37FCF4CD64F571883100</t>
+          <t>https://www.adzuna.in/land/ad/5750495104?se=Lq3IaR1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=BEB267C4FE33B892711F37FCF4CD64F571883100</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5749037378?se=nkMGsRRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=439C1013C31F64FF3D99143A4ABE4BA606CE0AEF</t>
+          <t>https://www.adzuna.in/land/ad/5749037378?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=439C1013C31F64FF3D99143A4ABE4BA606CE0AEF</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762133961?se=OEaUrhRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A567A465BBFA1F3725C3B40E702992E52F05EC45</t>
+          <t>https://www.adzuna.in/land/ad/5762133961?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A567A465BBFA1F3725C3B40E702992E52F05EC45</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5374790512?se=ciozsBRu8RGl0MKcaJBBpg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=161F0A4DE9F0D2B630015CA623E46D4A8B0D94E6</t>
+          <t>https://www.adzuna.in/land/ad/5374790512?se=Lq3IaR1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=161F0A4DE9F0D2B630015CA623E46D4A8B0D94E6</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279202?se=nkMGsRRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1DBB13C9620B1595275539972BC811719534C035</t>
+          <t>https://www.adzuna.in/land/ad/5769279202?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1DBB13C9620B1595275539972BC811719534C035</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5677690679?se=ciozsBRu8RGl0MKcaJBBpg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=075C0624B177AAAB43DA3F8D6FB39E63891EAFC6</t>
+          <t>https://www.adzuna.in/land/ad/5677690679?se=Lq3IaR1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=075C0624B177AAAB43DA3F8D6FB39E63891EAFC6</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5721567196?se=nkMGsRRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=CFA01DD69555B396E78C88671A3221E1D0E3A905</t>
+          <t>https://www.adzuna.in/land/ad/5721567196?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=CFA01DD69555B396E78C88671A3221E1D0E3A905</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017103?se=nkMGsRRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4F3763ADB1BAC8967835B18C3B88976D059CB89</t>
+          <t>https://www.adzuna.in/land/ad/5768017103?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4F3763ADB1BAC8967835B18C3B88976D059CB89</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762132173?se=OEaUrhRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4FD2F2920AB055E5DF8BA7C040CF14891EE744D5</t>
+          <t>https://www.adzuna.in/land/ad/5762132173?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4FD2F2920AB055E5DF8BA7C040CF14891EE744D5</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762136519?se=nkMGsRRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1C916FB5C4AD09CEE16D3473EE88C0A6B6F865BB</t>
+          <t>https://www.adzuna.in/land/ad/5762136519?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1C916FB5C4AD09CEE16D3473EE88C0A6B6F865BB</t>
         </is>
       </c>
     </row>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762134217?se=oFtmrxRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=146A7355AE9AC5AC172455EB2B0E549F081EEADA</t>
+          <t>https://www.adzuna.in/land/ad/5762134217?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=146A7355AE9AC5AC172455EB2B0E549F081EEADA</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753854807?se=nkMGsRRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6142203C924F3EE1A80E3E8335EA7AF45143A5C6</t>
+          <t>https://www.adzuna.in/land/ad/5753854807?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6142203C924F3EE1A80E3E8335EA7AF45143A5C6</t>
         </is>
       </c>
     </row>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768018385?se=nkMGsRRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1BF74BBEF1DAFDEE41395186E5489C69F4BEE8BC</t>
+          <t>https://www.adzuna.in/land/ad/5768018385?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1BF74BBEF1DAFDEE41395186E5489C69F4BEE8BC</t>
         </is>
       </c>
     </row>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745167451?se=ih_KsRRu8RGrKszqFbIEfQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1B7A588380034AAC42D886A7592B02CBF24E34A</t>
+          <t>https://www.adzuna.in/land/ad/5745167451?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1B7A588380034AAC42D886A7592B02CBF24E34A</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745166822?se=7OfVrRRu8RGnVKxb14Z7EQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=75DC13623E0BEA957F10FDAE9EDE19728AAF88FE</t>
+          <t>https://www.adzuna.in/land/ad/5745166822?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=75DC13623E0BEA957F10FDAE9EDE19728AAF88FE</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1889,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5737585201?se=nkMGsRRu8RGJe8gKxAvXaw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1E457E6EF8E102A87845B46934F33F96B5E3422</t>
+          <t>https://www.adzuna.in/land/ad/5737585201?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1E457E6EF8E102A87845B46934F33F96B5E3422</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AI Job Hunter v10.0 Status Management Dashboard
</commit_message>
<xml_diff>
--- a/output/jobs.xlsx
+++ b/output/jobs.xlsx
@@ -464,7 +464,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5743507343?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EC3CE217025746C9731AE4A3FE3C1282A6011BCA</t>
+          <t>https://www.adzuna.in/land/ad/5743507343?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EC3CE217025746C9731AE4A3FE3C1282A6011BCA</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5730011191?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=32B1BBCA420C902A6F2C3E09000395AA8FE6A3F5</t>
+          <t>https://www.adzuna.in/land/ad/5730011191?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=32B1BBCA420C902A6F2C3E09000395AA8FE6A3F5</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279977?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8140C4A63ACF7397C81D83F8A2E0D465705EC102</t>
+          <t>https://www.adzuna.in/land/ad/5769279977?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8140C4A63ACF7397C81D83F8A2E0D465705EC102</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742256993?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0C287C3961DC24298C835CB9417F8B09383F0052</t>
+          <t>https://www.adzuna.in/land/ad/5742256993?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0C287C3961DC24298C835CB9417F8B09383F0052</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763490875?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=F6580EC1E05F8A53AD05B2797EF5A9096F16DF5B</t>
+          <t>https://www.adzuna.in/land/ad/5763490875?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=F6580EC1E05F8A53AD05B2797EF5A9096F16DF5B</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763491420?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3FBB99E390EDF9FEBCE53C278A62FE4664A860EC</t>
+          <t>https://www.adzuna.in/land/ad/5763491420?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3FBB99E390EDF9FEBCE53C278A62FE4664A860EC</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742256422?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=511A44A56B34F4F4124473FA10BE5E077D5B6C3D</t>
+          <t>https://www.adzuna.in/land/ad/5742256422?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=511A44A56B34F4F4124473FA10BE5E077D5B6C3D</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017767?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1D57181F57C2D41E58572804A36F43C3D4AE9DD3</t>
+          <t>https://www.adzuna.in/land/ad/5768017767?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1D57181F57C2D41E58572804A36F43C3D4AE9DD3</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5751935354?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F393812E08FBC954B1FB55EE1B56E2DFB50954C</t>
+          <t>https://www.adzuna.in/land/ad/5751935354?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F393812E08FBC954B1FB55EE1B56E2DFB50954C</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747040297?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2E896599C4FAA7BFB268F9232FAAD133084B0921</t>
+          <t>https://www.adzuna.in/land/ad/5747040297?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2E896599C4FAA7BFB268F9232FAAD133084B0921</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753854888?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=DCC65B6F5A7A335BD330AF1C5879E10E1A0DA2BF</t>
+          <t>https://www.adzuna.in/land/ad/5753854888?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=DCC65B6F5A7A335BD330AF1C5879E10E1A0DA2BF</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762127810?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=55DA7A82770C696150F83F8133FACA98264C6E3F</t>
+          <t>https://www.adzuna.in/land/ad/5762127810?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=55DA7A82770C696150F83F8133FACA98264C6E3F</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5754995429?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=62BBB042D860B38D9BB38703AA92E62E26E7FEEF</t>
+          <t>https://www.adzuna.in/land/ad/5754995429?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=62BBB042D860B38D9BB38703AA92E62E26E7FEEF</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765773904?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=13B225115728D3657DA50775D7912A9BA4ED36EB</t>
+          <t>https://www.adzuna.in/land/ad/5765773904?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=13B225115728D3657DA50775D7912A9BA4ED36EB</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765771294?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=66B0C0764A60AE7A967A48E96A0935EBE89724C7</t>
+          <t>https://www.adzuna.in/land/ad/5765771294?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=66B0C0764A60AE7A967A48E96A0935EBE89724C7</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5697518505?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=9CEC78D19FCA0C7369A7A9F85A518FE1FD101D9B</t>
+          <t>https://www.adzuna.in/land/ad/5697518505?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=9CEC78D19FCA0C7369A7A9F85A518FE1FD101D9B</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753861658?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2FEC94CE5CB423BFE26CF6D30B22638EDBB7E8F1</t>
+          <t>https://www.adzuna.in/land/ad/5753861658?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2FEC94CE5CB423BFE26CF6D30B22638EDBB7E8F1</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017975?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=69D84AF1829A42AB98C8A52ADFD1EFCF7612FD49</t>
+          <t>https://www.adzuna.in/land/ad/5768017975?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=69D84AF1829A42AB98C8A52ADFD1EFCF7612FD49</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279314?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D58B4AE61A5DFD6033A10582B36518DC793AE0F4</t>
+          <t>https://www.adzuna.in/land/ad/5769279314?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D58B4AE61A5DFD6033A10582B36518DC793AE0F4</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5718579853?se=Lq3IaR1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EEB22977836DEAF81366ED7E9D416316985AA188</t>
+          <t>https://www.adzuna.in/land/ad/5718579853?se=JvgOpipu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EEB22977836DEAF81366ED7E9D416316985AA188</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5771700968?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=84E1AD6D342B54E01DADB5E011C6B186221EC596</t>
+          <t>https://www.adzuna.in/land/ad/5771700968?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=84E1AD6D342B54E01DADB5E011C6B186221EC596</t>
         </is>
       </c>
     </row>
@@ -989,7 +989,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753861185?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=764A0D94268C270F0A11F41CD71DC452D8D024EE</t>
+          <t>https://www.adzuna.in/land/ad/5753861185?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=764A0D94268C270F0A11F41CD71DC452D8D024EE</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765775462?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=37EF76F5E17E818F0447F6892E3D3033BCA9DEDB</t>
+          <t>https://www.adzuna.in/land/ad/5765775462?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=37EF76F5E17E818F0447F6892E3D3033BCA9DEDB</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747047144?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=086536F916DBD1B18D3DC8ADC94A41EDB4152A26</t>
+          <t>https://www.adzuna.in/land/ad/5747047144?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=086536F916DBD1B18D3DC8ADC94A41EDB4152A26</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5751935153?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=C4885E317E9A9D605051F18481BAC78ADCE69845</t>
+          <t>https://www.adzuna.in/land/ad/5751935153?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=C4885E317E9A9D605051F18481BAC78ADCE69845</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5750488988?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D508B9EDA6796D7FEA984502C190316CE8C2A72B</t>
+          <t>https://www.adzuna.in/land/ad/5750488988?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D508B9EDA6796D7FEA984502C190316CE8C2A72B</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5724225887?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=977640AFE7E1437C6FA9D94E36E92EE120B06CDA</t>
+          <t>https://www.adzuna.in/land/ad/5724225887?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=977640AFE7E1437C6FA9D94E36E92EE120B06CDA</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753195076?se=Lq3IaR1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=923801176AE7A1C9773F36AF178EBD26D512CA14</t>
+          <t>https://www.adzuna.in/land/ad/5753195076?se=JvgOpipu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=923801176AE7A1C9773F36AF178EBD26D512CA14</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763490809?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2DE9C024149D8DBE2A1313F30D55C8D54F432F3D</t>
+          <t>https://www.adzuna.in/land/ad/5763490809?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2DE9C024149D8DBE2A1313F30D55C8D54F432F3D</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765772430?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=E53BCFC3CB04BBEBC29296EC5F4B42289617F051</t>
+          <t>https://www.adzuna.in/land/ad/5765772430?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=E53BCFC3CB04BBEBC29296EC5F4B42289617F051</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742257007?se=Lq3IaR1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2D757BB48A163442E841856250996D40F30FC3E4</t>
+          <t>https://www.adzuna.in/land/ad/5742257007?se=JvgOpipu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2D757BB48A163442E841856250996D40F30FC3E4</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745164418?se=Lq3IaR1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3B0A759BCDB59AF4E25E85006C1AB1D0EB157057</t>
+          <t>https://www.adzuna.in/land/ad/5745164418?se=JvgOpipu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3B0A759BCDB59AF4E25E85006C1AB1D0EB157057</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5771700899?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EAC9690D3DACE0A8E1DB58475E6591E96A8C07DF</t>
+          <t>https://www.adzuna.in/land/ad/5771700899?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EAC9690D3DACE0A8E1DB58475E6591E96A8C07DF</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747049084?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=125E41A1B9DDB57408262D54D83632341383D0EB</t>
+          <t>https://www.adzuna.in/land/ad/5747049084?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=125E41A1B9DDB57408262D54D83632341383D0EB</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5760048697?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=70CA53C4D36C78E465CA1A70805E0139B2E3FFAB</t>
+          <t>https://www.adzuna.in/land/ad/5760048697?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=70CA53C4D36C78E465CA1A70805E0139B2E3FFAB</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5757284504?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=FBC032DA8BAD5D3101B3CC9E54E5B69521B6E72A</t>
+          <t>https://www.adzuna.in/land/ad/5757284504?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=FBC032DA8BAD5D3101B3CC9E54E5B69521B6E72A</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763491377?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4B3A4958BCF6866E580142C09980F0C770C32C7</t>
+          <t>https://www.adzuna.in/land/ad/5763491377?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4B3A4958BCF6866E580142C09980F0C770C32C7</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017288?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=83958946379D0B2DA69D00F6C975FEC5992724E7</t>
+          <t>https://www.adzuna.in/land/ad/5768017288?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=83958946379D0B2DA69D00F6C975FEC5992724E7</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753191970?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6BDA6CC2A00FC003582875F486E3C68BB692E1A3</t>
+          <t>https://www.adzuna.in/land/ad/5753191970?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6BDA6CC2A00FC003582875F486E3C68BB692E1A3</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5750495104?se=Lq3IaR1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=BEB267C4FE33B892711F37FCF4CD64F571883100</t>
+          <t>https://www.adzuna.in/land/ad/5750495104?se=JvgOpipu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=BEB267C4FE33B892711F37FCF4CD64F571883100</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5749037378?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=439C1013C31F64FF3D99143A4ABE4BA606CE0AEF</t>
+          <t>https://www.adzuna.in/land/ad/5749037378?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=439C1013C31F64FF3D99143A4ABE4BA606CE0AEF</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762133961?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A567A465BBFA1F3725C3B40E702992E52F05EC45</t>
+          <t>https://www.adzuna.in/land/ad/5762133961?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A567A465BBFA1F3725C3B40E702992E52F05EC45</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5374790512?se=Lq3IaR1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=161F0A4DE9F0D2B630015CA623E46D4A8B0D94E6</t>
+          <t>https://www.adzuna.in/land/ad/5374790512?se=JvgOpipu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=161F0A4DE9F0D2B630015CA623E46D4A8B0D94E6</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279202?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1DBB13C9620B1595275539972BC811719534C035</t>
+          <t>https://www.adzuna.in/land/ad/5769279202?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1DBB13C9620B1595275539972BC811719534C035</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5677690679?se=Lq3IaR1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=075C0624B177AAAB43DA3F8D6FB39E63891EAFC6</t>
+          <t>https://www.adzuna.in/land/ad/5677690679?se=JvgOpipu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=075C0624B177AAAB43DA3F8D6FB39E63891EAFC6</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5721567196?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=CFA01DD69555B396E78C88671A3221E1D0E3A905</t>
+          <t>https://www.adzuna.in/land/ad/5721567196?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=CFA01DD69555B396E78C88671A3221E1D0E3A905</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017103?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4F3763ADB1BAC8967835B18C3B88976D059CB89</t>
+          <t>https://www.adzuna.in/land/ad/5768017103?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4F3763ADB1BAC8967835B18C3B88976D059CB89</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762132173?se=eIgnaB1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4FD2F2920AB055E5DF8BA7C040CF14891EE744D5</t>
+          <t>https://www.adzuna.in/land/ad/5762132173?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4FD2F2920AB055E5DF8BA7C040CF14891EE744D5</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762136519?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1C916FB5C4AD09CEE16D3473EE88C0A6B6F865BB</t>
+          <t>https://www.adzuna.in/land/ad/5762136519?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1C916FB5C4AD09CEE16D3473EE88C0A6B6F865BB</t>
         </is>
       </c>
     </row>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762134217?se=-Ff1aB1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=146A7355AE9AC5AC172455EB2B0E549F081EEADA</t>
+          <t>https://www.adzuna.in/land/ad/5762134217?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=146A7355AE9AC5AC172455EB2B0E549F081EEADA</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753854807?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6142203C924F3EE1A80E3E8335EA7AF45143A5C6</t>
+          <t>https://www.adzuna.in/land/ad/5753854807?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6142203C924F3EE1A80E3E8335EA7AF45143A5C6</t>
         </is>
       </c>
     </row>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768018385?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1BF74BBEF1DAFDEE41395186E5489C69F4BEE8BC</t>
+          <t>https://www.adzuna.in/land/ad/5768018385?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1BF74BBEF1DAFDEE41395186E5489C69F4BEE8BC</t>
         </is>
       </c>
     </row>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745167451?se=ADRQax1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1B7A588380034AAC42D886A7592B02CBF24E34A</t>
+          <t>https://www.adzuna.in/land/ad/5745167451?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1B7A588380034AAC42D886A7592B02CBF24E34A</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745166822?se=qMtGZx1u8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=75DC13623E0BEA957F10FDAE9EDE19728AAF88FE</t>
+          <t>https://www.adzuna.in/land/ad/5745166822?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=75DC13623E0BEA957F10FDAE9EDE19728AAF88FE</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1889,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5737585201?se=HKOJah1u8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1E457E6EF8E102A87845B46934F33F96B5E3422</t>
+          <t>https://www.adzuna.in/land/ad/5737585201?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1E457E6EF8E102A87845B46934F33F96B5E3422</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AI Job Hunter v11.0 Stable
</commit_message>
<xml_diff>
--- a/output/jobs.xlsx
+++ b/output/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,7 +464,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5743507343?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EC3CE217025746C9731AE4A3FE3C1282A6011BCA</t>
+          <t>https://www.adzuna.in/land/ad/5743507343?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EC3CE217025746C9731AE4A3FE3C1282A6011BCA</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5730011191?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=32B1BBCA420C902A6F2C3E09000395AA8FE6A3F5</t>
+          <t>https://www.adzuna.in/land/ad/5730011191?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=32B1BBCA420C902A6F2C3E09000395AA8FE6A3F5</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279977?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8140C4A63ACF7397C81D83F8A2E0D465705EC102</t>
+          <t>https://www.adzuna.in/land/ad/5769279977?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8140C4A63ACF7397C81D83F8A2E0D465705EC102</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742256993?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0C287C3961DC24298C835CB9417F8B09383F0052</t>
+          <t>https://www.adzuna.in/land/ad/5742256993?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0C287C3961DC24298C835CB9417F8B09383F0052</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763490875?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=F6580EC1E05F8A53AD05B2797EF5A9096F16DF5B</t>
+          <t>https://www.adzuna.in/land/ad/5763490875?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=F6580EC1E05F8A53AD05B2797EF5A9096F16DF5B</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763491420?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3FBB99E390EDF9FEBCE53C278A62FE4664A860EC</t>
+          <t>https://www.adzuna.in/land/ad/5763491420?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3FBB99E390EDF9FEBCE53C278A62FE4664A860EC</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742256422?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=511A44A56B34F4F4124473FA10BE5E077D5B6C3D</t>
+          <t>https://www.adzuna.in/land/ad/5742256422?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=511A44A56B34F4F4124473FA10BE5E077D5B6C3D</t>
         </is>
       </c>
     </row>
@@ -639,144 +639,144 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017767?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1D57181F57C2D41E58572804A36F43C3D4AE9DD3</t>
+          <t>https://www.adzuna.in/land/ad/5768017767?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1D57181F57C2D41E58572804A36F43C3D4AE9DD3</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Network Engineer</t>
+          <t>Cyber Security Specialist</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Trantor</t>
+          <t>Adani Group</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>59.76</v>
+        <v>60.58</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5751935354?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F393812E08FBC954B1FB55EE1B56E2DFB50954C</t>
+          <t>https://www.adzuna.in/land/ad/5760051160?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=5E3C2778AFCF7D6B77821D7D853F7D93D646BD73</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Cyber Security Consultant</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Coforge</t>
+          <t>Trantor</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Delhi, India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>59.11</v>
+        <v>59.76</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747040297?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2E896599C4FAA7BFB268F9232FAAD133084B0921</t>
+          <t>https://www.adzuna.in/land/ad/5751935354?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F393812E08FBC954B1FB55EE1B56E2DFB50954C</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cyber Security Specialist</t>
+          <t>Cyber Security Consultant</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BuzzClan</t>
+          <t>Coforge</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Delhi, India</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>57.27</v>
+        <v>59.11</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753854888?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=DCC65B6F5A7A335BD330AF1C5879E10E1A0DA2BF</t>
+          <t>https://www.adzuna.in/land/ad/5747040297?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2E896599C4FAA7BFB268F9232FAAD133084B0921</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cyber Security Architect</t>
+          <t>Cyber Security Specialist</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tata Advanced Systems Limited</t>
+          <t>BuzzClan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Noida, Ghaziabad</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>56.25</v>
+        <v>57.27</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762127810?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=55DA7A82770C696150F83F8133FACA98264C6E3F</t>
+          <t>https://www.adzuna.in/land/ad/5753854888?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=DCC65B6F5A7A335BD330AF1C5879E10E1A0DA2BF</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cyber Security Engineer</t>
+          <t>Cyber Security Architect</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IntraEdge</t>
+          <t>Tata Advanced Systems Limited</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Noida, Ghaziabad</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>56.12</v>
+        <v>56.25</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5754995429?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=62BBB042D860B38D9BB38703AA92E62E26E7FEEF</t>
+          <t>https://www.adzuna.in/land/ad/5762127810?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=55DA7A82770C696150F83F8133FACA98264C6E3F</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Network Engineer</t>
+          <t>Cyber Security Engineer</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Coforge</t>
+          <t>IntraEdge</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -785,23 +785,23 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>55.7</v>
+        <v>56.12</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765773904?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=13B225115728D3657DA50775D7912A9BA4ED36EB</t>
+          <t>https://www.adzuna.in/land/ad/5754995429?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=62BBB042D860B38D9BB38703AA92E62E26E7FEEF</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SOC Detection and Automation engineer</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HCLSoftware</t>
+          <t>Coforge</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -810,248 +810,248 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>55.63</v>
+        <v>55.7</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765771294?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=66B0C0764A60AE7A967A48E96A0935EBE89724C7</t>
+          <t>https://www.adzuna.in/land/ad/5765773904?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=13B225115728D3657DA50775D7912A9BA4ED36EB</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Network Engineer</t>
+          <t>SOC Detection and Automation engineer</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Licious</t>
+          <t>HCLSoftware</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>54.92</v>
+        <v>55.63</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5697518505?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=9CEC78D19FCA0C7369A7A9F85A518FE1FD101D9B</t>
+          <t>https://www.adzuna.in/land/ad/5765771294?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=66B0C0764A60AE7A967A48E96A0935EBE89724C7</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Cyber Security Engineer</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Coforge</t>
+          <t>Licious</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Noida, Ghaziabad</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>54.74</v>
+        <v>54.92</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753861658?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2FEC94CE5CB423BFE26CF6D30B22638EDBB7E8F1</t>
+          <t>https://www.adzuna.in/land/ad/5697518505?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=9CEC78D19FCA0C7369A7A9F85A518FE1FD101D9B</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Information Security Analyst</t>
+          <t>Cyber Security Engineer</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HealthKart</t>
+          <t>Coforge</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Noida, Ghaziabad</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54.3</v>
+        <v>54.74</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017975?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=69D84AF1829A42AB98C8A52ADFD1EFCF7612FD49</t>
+          <t>https://www.adzuna.in/land/ad/5753861658?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2FEC94CE5CB423BFE26CF6D30B22638EDBB7E8F1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Cyber Security Analyst</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CenturyIQ</t>
+          <t>IH</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Thane, Maharashtra</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54.06</v>
+        <v>54.51</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279314?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D58B4AE61A5DFD6033A10582B36518DC793AE0F4</t>
+          <t>https://www.adzuna.in/land/ad/5773100081?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4E47ED62AE22E7EC84290A3E8AA04AC0672BE472</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Senior Network Engineer</t>
+          <t>Information Security Analyst</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>NEXPLAY SECURE</t>
+          <t>HealthKart</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>53.8</v>
+        <v>54.3</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5718579853?se=JvgOpipu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EEB22977836DEAF81366ED7E9D416316985AA188</t>
+          <t>https://www.adzuna.in/land/ad/5768017975?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=69D84AF1829A42AB98C8A52ADFD1EFCF7612FD49</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Cyber Security Trainer</t>
+          <t>Cyber Security Analyst</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Adani Skill Development Centre</t>
+          <t>CenturyIQ</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>53.35</v>
+        <v>54.06</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5771700968?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=84E1AD6D342B54E01DADB5E011C6B186221EC596</t>
+          <t>https://www.adzuna.in/land/ad/5769279314?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D58B4AE61A5DFD6033A10582B36518DC793AE0F4</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Network Engineer</t>
+          <t>Senior Network Engineer</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CloudFulcrum</t>
+          <t>NEXPLAY SECURE</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>53.28</v>
+        <v>53.8</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753861185?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=764A0D94268C270F0A11F41CD71DC452D8D024EE</t>
+          <t>https://www.adzuna.in/land/ad/5718579853?se=QiC0kLpu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EEB22977836DEAF81366ED7E9D416316985AA188</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Security Analyst</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Searce Inc</t>
+          <t>CloudFulcrum</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>52.43</v>
+        <v>53.28</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765775462?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=37EF76F5E17E818F0447F6892E3D3033BCA9DEDB</t>
+          <t>https://www.adzuna.in/land/ad/5753861185?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=764A0D94268C270F0A11F41CD71DC452D8D024EE</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Cyber Security Architect</t>
+          <t>Security Analyst</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AXISCADES</t>
+          <t>Searce Inc</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>51.91</v>
+        <v>52.43</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747047144?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=086536F916DBD1B18D3DC8ADC94A41EDB4152A26</t>
+          <t>https://www.adzuna.in/land/ad/5765775462?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=37EF76F5E17E818F0447F6892E3D3033BCA9DEDB</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Cyber Security Specialist</t>
+          <t>Cyber Security Architect</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ITC Infotech</t>
+          <t>AXISCADES</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1060,61 +1060,61 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>51.58</v>
+        <v>51.91</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5751935153?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=C4885E317E9A9D605051F18481BAC78ADCE69845</t>
+          <t>https://www.adzuna.in/land/ad/5747047144?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=086536F916DBD1B18D3DC8ADC94A41EDB4152A26</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>System Administrator</t>
+          <t>Cyber Security Specialist</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ACL Digital</t>
+          <t>ITC Infotech</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>50.72</v>
+        <v>51.58</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5750488988?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D508B9EDA6796D7FEA984502C190316CE8C2A72B</t>
+          <t>https://www.adzuna.in/land/ad/5751935153?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=C4885E317E9A9D605051F18481BAC78ADCE69845</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Network Engineer</t>
+          <t>System Administrator</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ServeMaison</t>
+          <t>ACL Digital</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>50.61</v>
+        <v>50.72</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5724225887?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=977640AFE7E1437C6FA9D94E36E92EE120B06CDA</t>
+          <t>https://www.adzuna.in/land/ad/5750488988?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D508B9EDA6796D7FEA984502C190316CE8C2A72B</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753195076?se=JvgOpipu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=923801176AE7A1C9773F36AF178EBD26D512CA14</t>
+          <t>https://www.adzuna.in/land/ad/5753195076?se=QiC0kLpu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=923801176AE7A1C9773F36AF178EBD26D512CA14</t>
         </is>
       </c>
     </row>
@@ -1164,119 +1164,119 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763490809?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2DE9C024149D8DBE2A1313F30D55C8D54F432F3D</t>
+          <t>https://www.adzuna.in/land/ad/5763490809?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2DE9C024149D8DBE2A1313F30D55C8D54F432F3D</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Senior Security Engineer</t>
+          <t>NOC Engineer (Admin)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GRIDsentry</t>
+          <t>Sonata Software</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>48.3</v>
+        <v>48.24</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765772430?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=E53BCFC3CB04BBEBC29296EC5F4B42289617F051</t>
+          <t>https://www.adzuna.in/land/ad/5742257007?se=QiC0kLpu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2D757BB48A163442E841856250996D40F30FC3E4</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>NOC Engineer (Admin)</t>
+          <t>System Network Administrator</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Sonata Software</t>
+          <t>Check Point Software</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>48.24</v>
+        <v>47.56</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742257007?se=JvgOpipu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2D757BB48A163442E841856250996D40F30FC3E4</t>
+          <t>https://www.adzuna.in/land/ad/5745164418?se=QiC0kLpu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3B0A759BCDB59AF4E25E85006C1AB1D0EB157057</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>System Network Administrator</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Check Point Software</t>
+          <t>Persistent Systems</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>47.56</v>
+        <v>47.01</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745164418?se=JvgOpipu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3B0A759BCDB59AF4E25E85006C1AB1D0EB157057</t>
+          <t>https://www.adzuna.in/land/ad/5747049084?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=125E41A1B9DDB57408262D54D83632341383D0EB</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Cloud security Analyst</t>
+          <t>Cyber Security Trainer</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Talentgigs</t>
+          <t>PenCap Institute of Excellence</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Chennai, Tamil Nadu</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>47.17</v>
+        <v>46.24</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5771700899?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EAC9690D3DACE0A8E1DB58475E6591E96A8C07DF</t>
+          <t>https://www.adzuna.in/land/ad/5760048697?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=70CA53C4D36C78E465CA1A70805E0139B2E3FFAB</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Network Engineer</t>
+          <t>System Administrator</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Persistent Systems</t>
+          <t>Stefanini Group</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1285,198 +1285,198 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>47.01</v>
+        <v>46.19</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747049084?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=125E41A1B9DDB57408262D54D83632341383D0EB</t>
+          <t>https://www.adzuna.in/land/ad/5757284504?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=FBC032DA8BAD5D3101B3CC9E54E5B69521B6E72A</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cyber Security Trainer</t>
+          <t>Data Security Analyst</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PenCap Institute of Excellence</t>
+          <t>Generac</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>46.24</v>
+        <v>46.17</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5760048697?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=70CA53C4D36C78E465CA1A70805E0139B2E3FFAB</t>
+          <t>https://www.adzuna.in/land/ad/5763491377?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4B3A4958BCF6866E580142C09980F0C770C32C7</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>System Administrator</t>
+          <t>Associate Director - Cyber Security</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Stefanini Group</t>
+          <t>Dexian India</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Chennai, Tamil Nadu</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>46.19</v>
+        <v>44.9</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5757284504?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=FBC032DA8BAD5D3101B3CC9E54E5B69521B6E72A</t>
+          <t>https://www.adzuna.in/land/ad/5768017288?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=83958946379D0B2DA69D00F6C975FEC5992724E7</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Data Security Analyst</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Generac</t>
+          <t>Movate</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Chennai, Tamil Nadu</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>46.17</v>
+        <v>44.81</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763491377?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4B3A4958BCF6866E580142C09980F0C770C32C7</t>
+          <t>https://www.adzuna.in/land/ad/5753191970?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6BDA6CC2A00FC003582875F486E3C68BB692E1A3</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Associate Director - Cyber Security</t>
+          <t>Assistant Architect – Liaisoning (Municipal Liaisoning)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Dexian India</t>
+          <t>Designo Architects</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu</t>
+          <t>Navi Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>44.9</v>
+        <v>44.2</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017288?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=83958946379D0B2DA69D00F6C975FEC5992724E7</t>
+          <t>https://www.adzuna.in/land/ad/5750495104?se=QiC0kLpu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=BEB267C4FE33B892711F37FCF4CD64F571883100</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Network Engineer</t>
+          <t>System Administrator</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Movate</t>
+          <t>Persistent Systems</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>44.81</v>
+        <v>43.97</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753191970?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6BDA6CC2A00FC003582875F486E3C68BB692E1A3</t>
+          <t>https://www.adzuna.in/land/ad/5749037378?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=439C1013C31F64FF3D99143A4ABE4BA606CE0AEF</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Assistant Architect – Liaisoning (Municipal Liaisoning)</t>
+          <t>Senior Product Designer</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Designo Architects</t>
+          <t>Unosecur</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Navi Mumbai, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>44.2</v>
+        <v>43.88</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5750495104?se=JvgOpipu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=BEB267C4FE33B892711F37FCF4CD64F571883100</t>
+          <t>https://www.adzuna.in/land/ad/5773098521?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=61A7EF41B5D62A47BAD748487EF4F5BACF71C292</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>System Administrator</t>
+          <t>Data Security Analyst</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Persistent Systems</t>
+          <t>NuSummit Cybersecurity</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>43.97</v>
+        <v>43.28</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5749037378?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=439C1013C31F64FF3D99143A4ABE4BA606CE0AEF</t>
+          <t>https://www.adzuna.in/land/ad/5762133961?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A567A465BBFA1F3725C3B40E702992E52F05EC45</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Data Security Analyst</t>
+          <t>NoC Verification Engineer</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>NuSummit Cybersecurity</t>
+          <t>ACL Digital</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1485,36 +1485,36 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>43.28</v>
+        <v>42.25</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762133961?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A567A465BBFA1F3725C3B40E702992E52F05EC45</t>
+          <t>https://www.adzuna.in/land/ad/5374790512?se=QiC0kLpu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=161F0A4DE9F0D2B630015CA623E46D4A8B0D94E6</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>NoC Verification Engineer</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ACL Digital</t>
+          <t>HCLTech</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Chennai, Tamil Nadu</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>42.25</v>
+        <v>40.27</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5374790512?se=JvgOpipu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=161F0A4DE9F0D2B630015CA623E46D4A8B0D94E6</t>
+          <t>https://www.adzuna.in/land/ad/5772526122?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0BA78F1159A331083EC3248C8E944199D331E6E4</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279202?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1DBB13C9620B1595275539972BC811719534C035</t>
+          <t>https://www.adzuna.in/land/ad/5769279202?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1DBB13C9620B1595275539972BC811719534C035</t>
         </is>
       </c>
     </row>
@@ -1589,19 +1589,19 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5677690679?se=JvgOpipu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=075C0624B177AAAB43DA3F8D6FB39E63891EAFC6</t>
+          <t>https://www.adzuna.in/land/ad/5677690679?se=QiC0kLpu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=075C0624B177AAAB43DA3F8D6FB39E63891EAFC6</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Systems Administrator</t>
+          <t>Cyber Security Analyst</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Scry AI</t>
+          <t>Tata Consultancy Services</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1610,61 +1610,61 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>37.85</v>
+        <v>37.99</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5721567196?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=CFA01DD69555B396E78C88671A3221E1D0E3A905</t>
+          <t>https://www.adzuna.in/land/ad/5757286370?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F0C30441DA6E0D475D1B92065ABBB9E1AD92023</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Linux System Administrator</t>
+          <t>Systems Administrator</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MGT-COMMERCE GmbH</t>
+          <t>Scry AI</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>37.8</v>
+        <v>37.85</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017103?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4F3763ADB1BAC8967835B18C3B88976D059CB89</t>
+          <t>https://www.adzuna.in/land/ad/5721567196?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=CFA01DD69555B396E78C88671A3221E1D0E3A905</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>NOC Engineer</t>
+          <t>Linux System Administrator</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Arrise Solutions  Pvt. Ltd</t>
+          <t>MGT-COMMERCE GmbH</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>35.76</v>
+        <v>37.8</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/details/5722234753?utm_medium=api&amp;utm_source=df095dcc</t>
+          <t>https://www.adzuna.in/land/ad/5768017103?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4F3763ADB1BAC8967835B18C3B88976D059CB89</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762132173?se=As2HpCpu8RGw6orMd6W2gw&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4FD2F2920AB055E5DF8BA7C040CF14891EE744D5</t>
+          <t>https://www.adzuna.in/land/ad/5762132173?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4FD2F2920AB055E5DF8BA7C040CF14891EE744D5</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762136519?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1C916FB5C4AD09CEE16D3473EE88C0A6B6F865BB</t>
+          <t>https://www.adzuna.in/land/ad/5762136519?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1C916FB5C4AD09CEE16D3473EE88C0A6B6F865BB</t>
         </is>
       </c>
     </row>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762134217?se=lrpLpSpu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=146A7355AE9AC5AC172455EB2B0E549F081EEADA</t>
+          <t>https://www.adzuna.in/land/ad/5762134217?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=146A7355AE9AC5AC172455EB2B0E549F081EEADA</t>
         </is>
       </c>
     </row>
@@ -1789,107 +1789,132 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753854807?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6142203C924F3EE1A80E3E8335EA7AF45143A5C6</t>
+          <t>https://www.adzuna.in/land/ad/5753854807?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6142203C924F3EE1A80E3E8335EA7AF45143A5C6</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>System Administrator</t>
+          <t>NOC Engineer</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Boutiqaat</t>
+          <t>Aeris Communications</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Noida, Ghaziabad</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>27.12</v>
+        <v>28.15</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768018385?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1BF74BBEF1DAFDEE41395186E5489C69F4BEE8BC</t>
+          <t>https://www.adzuna.in/details/5400411738?utm_medium=api&amp;utm_source=df095dcc</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>EVP Cyber Security</t>
+          <t>System Administrator</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>VISTRA</t>
+          <t>Boutiqaat</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>20.18</v>
+        <v>27.12</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745167451?se=-pScpypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1B7A588380034AAC42D886A7592B02CBF24E34A</t>
+          <t>https://www.adzuna.in/land/ad/5768018385?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1BF74BBEF1DAFDEE41395186E5489C69F4BEE8BC</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Cyber Incident Response Lead</t>
+          <t>EVP Cyber Security</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Owens &amp; Minor</t>
+          <t>VISTRA</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>11.92</v>
+        <v>20.18</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745166822?se=eimqoypu8RGG7YcE4aLLAA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=75DC13623E0BEA957F10FDAE9EDE19728AAF88FE</t>
+          <t>https://www.adzuna.in/land/ad/5745167451?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1B7A588380034AAC42D886A7592B02CBF24E34A</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>Cyber Incident Response Lead</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Owens &amp; Minor</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5745166822?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=75DC13623E0BEA957F10FDAE9EDE19728AAF88FE</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>Systems Administrator</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>Lexitas</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>Chennai, Tamil Nadu</t>
         </is>
       </c>
-      <c r="D59" t="n">
+      <c r="D60" t="n">
         <v>9.619999999999999</v>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.in/land/ad/5737585201?se=JijZpipu8RG-C6DUZsghXQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1E457E6EF8E102A87845B46934F33F96B5E3422</t>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/5737585201?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1E457E6EF8E102A87845B46934F33F96B5E3422</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AI Job Hunter v13.0 Watchlist Alerts
</commit_message>
<xml_diff>
--- a/output/jobs.xlsx
+++ b/output/jobs.xlsx
@@ -464,7 +464,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5743507343?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EC3CE217025746C9731AE4A3FE3C1282A6011BCA</t>
+          <t>https://www.adzuna.in/land/ad/5743507343?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EC3CE217025746C9731AE4A3FE3C1282A6011BCA</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5730011191?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=32B1BBCA420C902A6F2C3E09000395AA8FE6A3F5</t>
+          <t>https://www.adzuna.in/land/ad/5730011191?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=32B1BBCA420C902A6F2C3E09000395AA8FE6A3F5</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279977?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8140C4A63ACF7397C81D83F8A2E0D465705EC102</t>
+          <t>https://www.adzuna.in/land/ad/5769279977?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8140C4A63ACF7397C81D83F8A2E0D465705EC102</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742256993?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0C287C3961DC24298C835CB9417F8B09383F0052</t>
+          <t>https://www.adzuna.in/land/ad/5742256993?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0C287C3961DC24298C835CB9417F8B09383F0052</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763490875?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=F6580EC1E05F8A53AD05B2797EF5A9096F16DF5B</t>
+          <t>https://www.adzuna.in/land/ad/5763490875?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=F6580EC1E05F8A53AD05B2797EF5A9096F16DF5B</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763491420?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3FBB99E390EDF9FEBCE53C278A62FE4664A860EC</t>
+          <t>https://www.adzuna.in/land/ad/5763491420?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3FBB99E390EDF9FEBCE53C278A62FE4664A860EC</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742256422?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=511A44A56B34F4F4124473FA10BE5E077D5B6C3D</t>
+          <t>https://www.adzuna.in/land/ad/5742256422?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=511A44A56B34F4F4124473FA10BE5E077D5B6C3D</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017767?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1D57181F57C2D41E58572804A36F43C3D4AE9DD3</t>
+          <t>https://www.adzuna.in/land/ad/5768017767?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1D57181F57C2D41E58572804A36F43C3D4AE9DD3</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5760051160?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=5E3C2778AFCF7D6B77821D7D853F7D93D646BD73</t>
+          <t>https://www.adzuna.in/land/ad/5760051160?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=5E3C2778AFCF7D6B77821D7D853F7D93D646BD73</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5751935354?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F393812E08FBC954B1FB55EE1B56E2DFB50954C</t>
+          <t>https://www.adzuna.in/land/ad/5751935354?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F393812E08FBC954B1FB55EE1B56E2DFB50954C</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747040297?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2E896599C4FAA7BFB268F9232FAAD133084B0921</t>
+          <t>https://www.adzuna.in/land/ad/5747040297?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2E896599C4FAA7BFB268F9232FAAD133084B0921</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753854888?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=DCC65B6F5A7A335BD330AF1C5879E10E1A0DA2BF</t>
+          <t>https://www.adzuna.in/land/ad/5753854888?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=DCC65B6F5A7A335BD330AF1C5879E10E1A0DA2BF</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762127810?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=55DA7A82770C696150F83F8133FACA98264C6E3F</t>
+          <t>https://www.adzuna.in/land/ad/5762127810?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=55DA7A82770C696150F83F8133FACA98264C6E3F</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5754995429?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=62BBB042D860B38D9BB38703AA92E62E26E7FEEF</t>
+          <t>https://www.adzuna.in/land/ad/5754995429?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=62BBB042D860B38D9BB38703AA92E62E26E7FEEF</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765773904?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=13B225115728D3657DA50775D7912A9BA4ED36EB</t>
+          <t>https://www.adzuna.in/land/ad/5765773904?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=13B225115728D3657DA50775D7912A9BA4ED36EB</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765771294?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=66B0C0764A60AE7A967A48E96A0935EBE89724C7</t>
+          <t>https://www.adzuna.in/land/ad/5765771294?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=66B0C0764A60AE7A967A48E96A0935EBE89724C7</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5697518505?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=9CEC78D19FCA0C7369A7A9F85A518FE1FD101D9B</t>
+          <t>https://www.adzuna.in/land/ad/5697518505?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=9CEC78D19FCA0C7369A7A9F85A518FE1FD101D9B</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753861658?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2FEC94CE5CB423BFE26CF6D30B22638EDBB7E8F1</t>
+          <t>https://www.adzuna.in/land/ad/5753861658?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2FEC94CE5CB423BFE26CF6D30B22638EDBB7E8F1</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5773100081?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4E47ED62AE22E7EC84290A3E8AA04AC0672BE472</t>
+          <t>https://www.adzuna.in/land/ad/5773100081?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4E47ED62AE22E7EC84290A3E8AA04AC0672BE472</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017975?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=69D84AF1829A42AB98C8A52ADFD1EFCF7612FD49</t>
+          <t>https://www.adzuna.in/land/ad/5768017975?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=69D84AF1829A42AB98C8A52ADFD1EFCF7612FD49</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279314?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D58B4AE61A5DFD6033A10582B36518DC793AE0F4</t>
+          <t>https://www.adzuna.in/land/ad/5769279314?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D58B4AE61A5DFD6033A10582B36518DC793AE0F4</t>
         </is>
       </c>
     </row>
@@ -989,7 +989,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5718579853?se=QiC0kLpu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EEB22977836DEAF81366ED7E9D416316985AA188</t>
+          <t>https://www.adzuna.in/land/ad/5718579853?se=YHRJlb1u8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EEB22977836DEAF81366ED7E9D416316985AA188</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753861185?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=764A0D94268C270F0A11F41CD71DC452D8D024EE</t>
+          <t>https://www.adzuna.in/land/ad/5753861185?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=764A0D94268C270F0A11F41CD71DC452D8D024EE</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765775462?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=37EF76F5E17E818F0447F6892E3D3033BCA9DEDB</t>
+          <t>https://www.adzuna.in/land/ad/5765775462?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=37EF76F5E17E818F0447F6892E3D3033BCA9DEDB</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747047144?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=086536F916DBD1B18D3DC8ADC94A41EDB4152A26</t>
+          <t>https://www.adzuna.in/land/ad/5747047144?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=086536F916DBD1B18D3DC8ADC94A41EDB4152A26</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5751935153?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=C4885E317E9A9D605051F18481BAC78ADCE69845</t>
+          <t>https://www.adzuna.in/land/ad/5751935153?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=C4885E317E9A9D605051F18481BAC78ADCE69845</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5750488988?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D508B9EDA6796D7FEA984502C190316CE8C2A72B</t>
+          <t>https://www.adzuna.in/land/ad/5750488988?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D508B9EDA6796D7FEA984502C190316CE8C2A72B</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753195076?se=QiC0kLpu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=923801176AE7A1C9773F36AF178EBD26D512CA14</t>
+          <t>https://www.adzuna.in/land/ad/5753195076?se=YHRJlb1u8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=923801176AE7A1C9773F36AF178EBD26D512CA14</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763490809?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2DE9C024149D8DBE2A1313F30D55C8D54F432F3D</t>
+          <t>https://www.adzuna.in/land/ad/5763490809?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2DE9C024149D8DBE2A1313F30D55C8D54F432F3D</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742257007?se=QiC0kLpu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2D757BB48A163442E841856250996D40F30FC3E4</t>
+          <t>https://www.adzuna.in/land/ad/5742257007?se=YHRJlb1u8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2D757BB48A163442E841856250996D40F30FC3E4</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745164418?se=QiC0kLpu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3B0A759BCDB59AF4E25E85006C1AB1D0EB157057</t>
+          <t>https://www.adzuna.in/land/ad/5745164418?se=YHRJlb1u8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3B0A759BCDB59AF4E25E85006C1AB1D0EB157057</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747049084?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=125E41A1B9DDB57408262D54D83632341383D0EB</t>
+          <t>https://www.adzuna.in/land/ad/5747049084?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=125E41A1B9DDB57408262D54D83632341383D0EB</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5760048697?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=70CA53C4D36C78E465CA1A70805E0139B2E3FFAB</t>
+          <t>https://www.adzuna.in/land/ad/5760048697?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=70CA53C4D36C78E465CA1A70805E0139B2E3FFAB</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5757284504?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=FBC032DA8BAD5D3101B3CC9E54E5B69521B6E72A</t>
+          <t>https://www.adzuna.in/land/ad/5757284504?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=FBC032DA8BAD5D3101B3CC9E54E5B69521B6E72A</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763491377?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4B3A4958BCF6866E580142C09980F0C770C32C7</t>
+          <t>https://www.adzuna.in/land/ad/5763491377?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4B3A4958BCF6866E580142C09980F0C770C32C7</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017288?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=83958946379D0B2DA69D00F6C975FEC5992724E7</t>
+          <t>https://www.adzuna.in/land/ad/5768017288?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=83958946379D0B2DA69D00F6C975FEC5992724E7</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753191970?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6BDA6CC2A00FC003582875F486E3C68BB692E1A3</t>
+          <t>https://www.adzuna.in/land/ad/5753191970?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6BDA6CC2A00FC003582875F486E3C68BB692E1A3</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5750495104?se=QiC0kLpu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=BEB267C4FE33B892711F37FCF4CD64F571883100</t>
+          <t>https://www.adzuna.in/land/ad/5750495104?se=YHRJlb1u8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=BEB267C4FE33B892711F37FCF4CD64F571883100</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5749037378?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=439C1013C31F64FF3D99143A4ABE4BA606CE0AEF</t>
+          <t>https://www.adzuna.in/land/ad/5749037378?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=439C1013C31F64FF3D99143A4ABE4BA606CE0AEF</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5773098521?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=61A7EF41B5D62A47BAD748487EF4F5BACF71C292</t>
+          <t>https://www.adzuna.in/land/ad/5773098521?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=61A7EF41B5D62A47BAD748487EF4F5BACF71C292</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762133961?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A567A465BBFA1F3725C3B40E702992E52F05EC45</t>
+          <t>https://www.adzuna.in/land/ad/5762133961?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A567A465BBFA1F3725C3B40E702992E52F05EC45</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5374790512?se=QiC0kLpu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=161F0A4DE9F0D2B630015CA623E46D4A8B0D94E6</t>
+          <t>https://www.adzuna.in/land/ad/5374790512?se=YHRJlb1u8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=161F0A4DE9F0D2B630015CA623E46D4A8B0D94E6</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5772526122?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0BA78F1159A331083EC3248C8E944199D331E6E4</t>
+          <t>https://www.adzuna.in/land/ad/5772526122?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0BA78F1159A331083EC3248C8E944199D331E6E4</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279202?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1DBB13C9620B1595275539972BC811719534C035</t>
+          <t>https://www.adzuna.in/land/ad/5769279202?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1DBB13C9620B1595275539972BC811719534C035</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5677690679?se=QiC0kLpu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=075C0624B177AAAB43DA3F8D6FB39E63891EAFC6</t>
+          <t>https://www.adzuna.in/land/ad/5677690679?se=YHRJlb1u8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=075C0624B177AAAB43DA3F8D6FB39E63891EAFC6</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5757286370?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F0C30441DA6E0D475D1B92065ABBB9E1AD92023</t>
+          <t>https://www.adzuna.in/land/ad/5757286370?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F0C30441DA6E0D475D1B92065ABBB9E1AD92023</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5721567196?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=CFA01DD69555B396E78C88671A3221E1D0E3A905</t>
+          <t>https://www.adzuna.in/land/ad/5721567196?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=CFA01DD69555B396E78C88671A3221E1D0E3A905</t>
         </is>
       </c>
     </row>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017103?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4F3763ADB1BAC8967835B18C3B88976D059CB89</t>
+          <t>https://www.adzuna.in/land/ad/5768017103?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4F3763ADB1BAC8967835B18C3B88976D059CB89</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762132173?se=1ocjj7pu8RGCk400RXzHVQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4FD2F2920AB055E5DF8BA7C040CF14891EE744D5</t>
+          <t>https://www.adzuna.in/land/ad/5762132173?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4FD2F2920AB055E5DF8BA7C040CF14891EE744D5</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762136519?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1C916FB5C4AD09CEE16D3473EE88C0A6B6F865BB</t>
+          <t>https://www.adzuna.in/land/ad/5762136519?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1C916FB5C4AD09CEE16D3473EE88C0A6B6F865BB</t>
         </is>
       </c>
     </row>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762134217?se=Xtzrj7pu8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=146A7355AE9AC5AC172455EB2B0E549F081EEADA</t>
+          <t>https://www.adzuna.in/land/ad/5762134217?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=146A7355AE9AC5AC172455EB2B0E549F081EEADA</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753854807?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6142203C924F3EE1A80E3E8335EA7AF45143A5C6</t>
+          <t>https://www.adzuna.in/land/ad/5753854807?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6142203C924F3EE1A80E3E8335EA7AF45143A5C6</t>
         </is>
       </c>
     </row>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768018385?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1BF74BBEF1DAFDEE41395186E5489C69F4BEE8BC</t>
+          <t>https://www.adzuna.in/land/ad/5768018385?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1BF74BBEF1DAFDEE41395186E5489C69F4BEE8BC</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745167451?se=xARMkrpu8RGIQNcU7oP5Ww&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1B7A588380034AAC42D886A7592B02CBF24E34A</t>
+          <t>https://www.adzuna.in/land/ad/5745167451?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1B7A588380034AAC42D886A7592B02CBF24E34A</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1889,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745166822?se=TO5ljrpu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=75DC13623E0BEA957F10FDAE9EDE19728AAF88FE</t>
+          <t>https://www.adzuna.in/land/ad/5745166822?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=75DC13623E0BEA957F10FDAE9EDE19728AAF88FE</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5737585201?se=_paAkbpu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1E457E6EF8E102A87845B46934F33F96B5E3422</t>
+          <t>https://www.adzuna.in/land/ad/5737585201?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1E457E6EF8E102A87845B46934F33F96B5E3422</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v15 Weekly PDF Reports
</commit_message>
<xml_diff>
--- a/output/jobs.xlsx
+++ b/output/jobs.xlsx
@@ -464,7 +464,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5743507343?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EC3CE217025746C9731AE4A3FE3C1282A6011BCA</t>
+          <t>https://www.adzuna.in/land/ad/5743507343?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EC3CE217025746C9731AE4A3FE3C1282A6011BCA</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5730011191?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=32B1BBCA420C902A6F2C3E09000395AA8FE6A3F5</t>
+          <t>https://www.adzuna.in/land/ad/5730011191?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=32B1BBCA420C902A6F2C3E09000395AA8FE6A3F5</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279977?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8140C4A63ACF7397C81D83F8A2E0D465705EC102</t>
+          <t>https://www.adzuna.in/land/ad/5769279977?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8140C4A63ACF7397C81D83F8A2E0D465705EC102</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742256993?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0C287C3961DC24298C835CB9417F8B09383F0052</t>
+          <t>https://www.adzuna.in/land/ad/5742256993?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0C287C3961DC24298C835CB9417F8B09383F0052</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763490875?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=F6580EC1E05F8A53AD05B2797EF5A9096F16DF5B</t>
+          <t>https://www.adzuna.in/land/ad/5763490875?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=F6580EC1E05F8A53AD05B2797EF5A9096F16DF5B</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763491420?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3FBB99E390EDF9FEBCE53C278A62FE4664A860EC</t>
+          <t>https://www.adzuna.in/land/ad/5763491420?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3FBB99E390EDF9FEBCE53C278A62FE4664A860EC</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742256422?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=511A44A56B34F4F4124473FA10BE5E077D5B6C3D</t>
+          <t>https://www.adzuna.in/land/ad/5742256422?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=511A44A56B34F4F4124473FA10BE5E077D5B6C3D</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017767?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1D57181F57C2D41E58572804A36F43C3D4AE9DD3</t>
+          <t>https://www.adzuna.in/land/ad/5768017767?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1D57181F57C2D41E58572804A36F43C3D4AE9DD3</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5760051160?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=5E3C2778AFCF7D6B77821D7D853F7D93D646BD73</t>
+          <t>https://www.adzuna.in/land/ad/5760051160?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=5E3C2778AFCF7D6B77821D7D853F7D93D646BD73</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5751935354?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F393812E08FBC954B1FB55EE1B56E2DFB50954C</t>
+          <t>https://www.adzuna.in/land/ad/5751935354?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F393812E08FBC954B1FB55EE1B56E2DFB50954C</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747040297?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2E896599C4FAA7BFB268F9232FAAD133084B0921</t>
+          <t>https://www.adzuna.in/land/ad/5747040297?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2E896599C4FAA7BFB268F9232FAAD133084B0921</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753854888?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=DCC65B6F5A7A335BD330AF1C5879E10E1A0DA2BF</t>
+          <t>https://www.adzuna.in/land/ad/5753854888?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=DCC65B6F5A7A335BD330AF1C5879E10E1A0DA2BF</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762127810?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=55DA7A82770C696150F83F8133FACA98264C6E3F</t>
+          <t>https://www.adzuna.in/land/ad/5762127810?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=55DA7A82770C696150F83F8133FACA98264C6E3F</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5754995429?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=62BBB042D860B38D9BB38703AA92E62E26E7FEEF</t>
+          <t>https://www.adzuna.in/land/ad/5754995429?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=62BBB042D860B38D9BB38703AA92E62E26E7FEEF</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765773904?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=13B225115728D3657DA50775D7912A9BA4ED36EB</t>
+          <t>https://www.adzuna.in/land/ad/5765773904?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=13B225115728D3657DA50775D7912A9BA4ED36EB</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765771294?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=66B0C0764A60AE7A967A48E96A0935EBE89724C7</t>
+          <t>https://www.adzuna.in/land/ad/5765771294?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=66B0C0764A60AE7A967A48E96A0935EBE89724C7</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5697518505?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=9CEC78D19FCA0C7369A7A9F85A518FE1FD101D9B</t>
+          <t>https://www.adzuna.in/land/ad/5697518505?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=9CEC78D19FCA0C7369A7A9F85A518FE1FD101D9B</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753861658?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2FEC94CE5CB423BFE26CF6D30B22638EDBB7E8F1</t>
+          <t>https://www.adzuna.in/land/ad/5753861658?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2FEC94CE5CB423BFE26CF6D30B22638EDBB7E8F1</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5773100081?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4E47ED62AE22E7EC84290A3E8AA04AC0672BE472</t>
+          <t>https://www.adzuna.in/land/ad/5773100081?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4E47ED62AE22E7EC84290A3E8AA04AC0672BE472</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017975?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=69D84AF1829A42AB98C8A52ADFD1EFCF7612FD49</t>
+          <t>https://www.adzuna.in/land/ad/5768017975?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=69D84AF1829A42AB98C8A52ADFD1EFCF7612FD49</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279314?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D58B4AE61A5DFD6033A10582B36518DC793AE0F4</t>
+          <t>https://www.adzuna.in/land/ad/5769279314?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D58B4AE61A5DFD6033A10582B36518DC793AE0F4</t>
         </is>
       </c>
     </row>
@@ -989,7 +989,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5718579853?se=YHRJlb1u8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EEB22977836DEAF81366ED7E9D416316985AA188</t>
+          <t>https://www.adzuna.in/land/ad/5718579853?se=miSUf8tu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EEB22977836DEAF81366ED7E9D416316985AA188</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753861185?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=764A0D94268C270F0A11F41CD71DC452D8D024EE</t>
+          <t>https://www.adzuna.in/land/ad/5753861185?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=764A0D94268C270F0A11F41CD71DC452D8D024EE</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765775462?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=37EF76F5E17E818F0447F6892E3D3033BCA9DEDB</t>
+          <t>https://www.adzuna.in/land/ad/5765775462?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=37EF76F5E17E818F0447F6892E3D3033BCA9DEDB</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747047144?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=086536F916DBD1B18D3DC8ADC94A41EDB4152A26</t>
+          <t>https://www.adzuna.in/land/ad/5747047144?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=086536F916DBD1B18D3DC8ADC94A41EDB4152A26</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5751935153?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=C4885E317E9A9D605051F18481BAC78ADCE69845</t>
+          <t>https://www.adzuna.in/land/ad/5751935153?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=C4885E317E9A9D605051F18481BAC78ADCE69845</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5750488988?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D508B9EDA6796D7FEA984502C190316CE8C2A72B</t>
+          <t>https://www.adzuna.in/land/ad/5750488988?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D508B9EDA6796D7FEA984502C190316CE8C2A72B</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753195076?se=YHRJlb1u8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=923801176AE7A1C9773F36AF178EBD26D512CA14</t>
+          <t>https://www.adzuna.in/land/ad/5753195076?se=miSUf8tu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=923801176AE7A1C9773F36AF178EBD26D512CA14</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763490809?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2DE9C024149D8DBE2A1313F30D55C8D54F432F3D</t>
+          <t>https://www.adzuna.in/land/ad/5763490809?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2DE9C024149D8DBE2A1313F30D55C8D54F432F3D</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742257007?se=YHRJlb1u8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2D757BB48A163442E841856250996D40F30FC3E4</t>
+          <t>https://www.adzuna.in/land/ad/5742257007?se=miSUf8tu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2D757BB48A163442E841856250996D40F30FC3E4</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745164418?se=YHRJlb1u8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3B0A759BCDB59AF4E25E85006C1AB1D0EB157057</t>
+          <t>https://www.adzuna.in/land/ad/5745164418?se=miSUf8tu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3B0A759BCDB59AF4E25E85006C1AB1D0EB157057</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747049084?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=125E41A1B9DDB57408262D54D83632341383D0EB</t>
+          <t>https://www.adzuna.in/land/ad/5747049084?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=125E41A1B9DDB57408262D54D83632341383D0EB</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5760048697?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=70CA53C4D36C78E465CA1A70805E0139B2E3FFAB</t>
+          <t>https://www.adzuna.in/land/ad/5760048697?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=70CA53C4D36C78E465CA1A70805E0139B2E3FFAB</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5757284504?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=FBC032DA8BAD5D3101B3CC9E54E5B69521B6E72A</t>
+          <t>https://www.adzuna.in/land/ad/5757284504?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=FBC032DA8BAD5D3101B3CC9E54E5B69521B6E72A</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763491377?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4B3A4958BCF6866E580142C09980F0C770C32C7</t>
+          <t>https://www.adzuna.in/land/ad/5763491377?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4B3A4958BCF6866E580142C09980F0C770C32C7</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017288?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=83958946379D0B2DA69D00F6C975FEC5992724E7</t>
+          <t>https://www.adzuna.in/land/ad/5768017288?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=83958946379D0B2DA69D00F6C975FEC5992724E7</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753191970?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6BDA6CC2A00FC003582875F486E3C68BB692E1A3</t>
+          <t>https://www.adzuna.in/land/ad/5753191970?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6BDA6CC2A00FC003582875F486E3C68BB692E1A3</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5750495104?se=YHRJlb1u8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=BEB267C4FE33B892711F37FCF4CD64F571883100</t>
+          <t>https://www.adzuna.in/land/ad/5750495104?se=miSUf8tu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=BEB267C4FE33B892711F37FCF4CD64F571883100</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5749037378?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=439C1013C31F64FF3D99143A4ABE4BA606CE0AEF</t>
+          <t>https://www.adzuna.in/land/ad/5749037378?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=439C1013C31F64FF3D99143A4ABE4BA606CE0AEF</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5773098521?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=61A7EF41B5D62A47BAD748487EF4F5BACF71C292</t>
+          <t>https://www.adzuna.in/land/ad/5773098521?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=61A7EF41B5D62A47BAD748487EF4F5BACF71C292</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762133961?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A567A465BBFA1F3725C3B40E702992E52F05EC45</t>
+          <t>https://www.adzuna.in/land/ad/5762133961?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A567A465BBFA1F3725C3B40E702992E52F05EC45</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5374790512?se=YHRJlb1u8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=161F0A4DE9F0D2B630015CA623E46D4A8B0D94E6</t>
+          <t>https://www.adzuna.in/land/ad/5374790512?se=miSUf8tu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=161F0A4DE9F0D2B630015CA623E46D4A8B0D94E6</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5772526122?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0BA78F1159A331083EC3248C8E944199D331E6E4</t>
+          <t>https://www.adzuna.in/land/ad/5772526122?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0BA78F1159A331083EC3248C8E944199D331E6E4</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279202?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1DBB13C9620B1595275539972BC811719534C035</t>
+          <t>https://www.adzuna.in/land/ad/5769279202?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1DBB13C9620B1595275539972BC811719534C035</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5677690679?se=YHRJlb1u8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=075C0624B177AAAB43DA3F8D6FB39E63891EAFC6</t>
+          <t>https://www.adzuna.in/land/ad/5677690679?se=miSUf8tu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=075C0624B177AAAB43DA3F8D6FB39E63891EAFC6</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5757286370?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F0C30441DA6E0D475D1B92065ABBB9E1AD92023</t>
+          <t>https://www.adzuna.in/land/ad/5757286370?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F0C30441DA6E0D475D1B92065ABBB9E1AD92023</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5721567196?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=CFA01DD69555B396E78C88671A3221E1D0E3A905</t>
+          <t>https://www.adzuna.in/land/ad/5721567196?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=CFA01DD69555B396E78C88671A3221E1D0E3A905</t>
         </is>
       </c>
     </row>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017103?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4F3763ADB1BAC8967835B18C3B88976D059CB89</t>
+          <t>https://www.adzuna.in/land/ad/5768017103?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4F3763ADB1BAC8967835B18C3B88976D059CB89</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762132173?se=qIgXk71u8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4FD2F2920AB055E5DF8BA7C040CF14891EE744D5</t>
+          <t>https://www.adzuna.in/land/ad/5762132173?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4FD2F2920AB055E5DF8BA7C040CF14891EE744D5</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762136519?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1C916FB5C4AD09CEE16D3473EE88C0A6B6F865BB</t>
+          <t>https://www.adzuna.in/land/ad/5762136519?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1C916FB5C4AD09CEE16D3473EE88C0A6B6F865BB</t>
         </is>
       </c>
     </row>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762134217?se=uPQ6lL1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=146A7355AE9AC5AC172455EB2B0E549F081EEADA</t>
+          <t>https://www.adzuna.in/land/ad/5762134217?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=146A7355AE9AC5AC172455EB2B0E549F081EEADA</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753854807?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6142203C924F3EE1A80E3E8335EA7AF45143A5C6</t>
+          <t>https://www.adzuna.in/land/ad/5753854807?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6142203C924F3EE1A80E3E8335EA7AF45143A5C6</t>
         </is>
       </c>
     </row>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768018385?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1BF74BBEF1DAFDEE41395186E5489C69F4BEE8BC</t>
+          <t>https://www.adzuna.in/land/ad/5768018385?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1BF74BBEF1DAFDEE41395186E5489C69F4BEE8BC</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745167451?se=tAfelr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1B7A588380034AAC42D886A7592B02CBF24E34A</t>
+          <t>https://www.adzuna.in/land/ad/5745167451?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1B7A588380034AAC42D886A7592B02CBF24E34A</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1889,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745166822?se=NP9bkr1u8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=75DC13623E0BEA957F10FDAE9EDE19728AAF88FE</t>
+          <t>https://www.adzuna.in/land/ad/5745166822?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=75DC13623E0BEA957F10FDAE9EDE19728AAF88FE</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5737585201?se=3BYblr1u8RGeWZzv8P2X6w&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1E457E6EF8E102A87845B46934F33F96B5E3422</t>
+          <t>https://www.adzuna.in/land/ad/5737585201?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1E457E6EF8E102A87845B46934F33F96B5E3422</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v18.1 Career Coach Intelligence
</commit_message>
<xml_diff>
--- a/output/jobs.xlsx
+++ b/output/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,362 +446,362 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Security Analyst</t>
+          <t>Network Security Engineer (IDS Operations)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Eventus Security</t>
+          <t>IH</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>70.15000000000001</v>
+        <v>72.12</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5743507343?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EC3CE217025746C9731AE4A3FE3C1282A6011BCA</t>
+          <t>https://www.adzuna.in/land/ad/5773100210?se=zvWGXeFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=F3C64941F91C760316D15431DF90B68265D330DB</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Security Engineer</t>
+          <t>Security Analyst</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>H&amp;R Block India</t>
+          <t>Eventus Security</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>68.22</v>
+        <v>70.15000000000001</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5730011191?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=32B1BBCA420C902A6F2C3E09000395AA8FE6A3F5</t>
+          <t>https://www.adzuna.in/land/ad/5743507343?se=zvWGXeFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EC3CE217025746C9731AE4A3FE3C1282A6011BCA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cyber Security Analyst</t>
+          <t>Security Engineer</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Vensure Employer Solutions</t>
+          <t>H&amp;R Block India</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thiruvananthapuram, Kerala</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>67</v>
+        <v>68.22</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279977?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8140C4A63ACF7397C81D83F8A2E0D465705EC102</t>
+          <t>https://www.adzuna.in/land/ad/5730011191?se=zvWGXeFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=32B1BBCA420C902A6F2C3E09000395AA8FE6A3F5</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SOC Manager</t>
+          <t>Cyber Security Analyst</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>C3iHub, IIT Kanpur</t>
+          <t>Vensure Employer Solutions</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Delhi, India</t>
+          <t>Thiruvananthapuram, Kerala</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>66.56999999999999</v>
+        <v>67</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742256993?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0C287C3961DC24298C835CB9417F8B09383F0052</t>
+          <t>https://www.adzuna.in/land/ad/5769279977?se=TOhCXuFu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8140C4A63ACF7397C81D83F8A2E0D465705EC102</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Senior Security Engineer</t>
+          <t>SOC Manager</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Eventus Security</t>
+          <t>C3iHub, IIT Kanpur</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Navi Mumbai, Maharashtra</t>
+          <t>Delhi, India</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>65.25</v>
+        <v>66.56999999999999</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763490875?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=F6580EC1E05F8A53AD05B2797EF5A9096F16DF5B</t>
+          <t>https://www.adzuna.in/land/ad/5742256993?se=zvWGXeFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0C287C3961DC24298C835CB9417F8B09383F0052</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Information Security Analyst</t>
+          <t>Senior Security Engineer</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EvonSys</t>
+          <t>Eventus Security</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Navi Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>64.76000000000001</v>
+        <v>65.25</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763491420?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3FBB99E390EDF9FEBCE53C278A62FE4664A860EC</t>
+          <t>https://www.adzuna.in/land/ad/5763490875?se=zvWGXeFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=F6580EC1E05F8A53AD05B2797EF5A9096F16DF5B</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Security Engineer - L2 (Immediate Joiner)</t>
+          <t>Information Security Analyst</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SHI Solutions India Pvt. Ltd.</t>
+          <t>EvonSys</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>62.51</v>
+        <v>64.76000000000001</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742256422?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=511A44A56B34F4F4124473FA10BE5E077D5B6C3D</t>
+          <t>https://www.adzuna.in/land/ad/5763491420?se=TOhCXuFu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3FBB99E390EDF9FEBCE53C278A62FE4664A860EC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cyber Security Lead</t>
+          <t>Security Engineer - L2 (Immediate Joiner)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TAC Security</t>
+          <t>SHI Solutions India Pvt. Ltd.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Chandigarh, India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>60.67</v>
+        <v>62.51</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017767?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1D57181F57C2D41E58572804A36F43C3D4AE9DD3</t>
+          <t>https://www.adzuna.in/land/ad/5742256422?se=zvWGXeFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=511A44A56B34F4F4124473FA10BE5E077D5B6C3D</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cyber Security Specialist</t>
+          <t>Cyber Security Lead</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Adani Group</t>
+          <t>TAC Security</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>Chandigarh, India</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>60.58</v>
+        <v>60.67</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5760051160?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=5E3C2778AFCF7D6B77821D7D853F7D93D646BD73</t>
+          <t>https://www.adzuna.in/land/ad/5768017767?se=QHteYeFu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1D57181F57C2D41E58572804A36F43C3D4AE9DD3</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Network Engineer</t>
+          <t>Cyber Security Specialist</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Trantor</t>
+          <t>Adani Group</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>59.76</v>
+        <v>60.58</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5751935354?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F393812E08FBC954B1FB55EE1B56E2DFB50954C</t>
+          <t>https://www.adzuna.in/land/ad/5760051160?se=QHteYeFu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=5E3C2778AFCF7D6B77821D7D853F7D93D646BD73</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cyber Security Consultant</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Coforge</t>
+          <t>Trantor</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Delhi, India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>59.11</v>
+        <v>59.76</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747040297?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2E896599C4FAA7BFB268F9232FAAD133084B0921</t>
+          <t>https://www.adzuna.in/land/ad/5751935354?se=hAEKX-Fu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F393812E08FBC954B1FB55EE1B56E2DFB50954C</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cyber Security Specialist</t>
+          <t>Cyber Security Consultant</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BuzzClan</t>
+          <t>Coforge</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Delhi, India</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>57.27</v>
+        <v>59.11</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753854888?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=DCC65B6F5A7A335BD330AF1C5879E10E1A0DA2BF</t>
+          <t>https://www.adzuna.in/land/ad/5747040297?se=QHteYeFu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2E896599C4FAA7BFB268F9232FAAD133084B0921</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cyber Security Architect</t>
+          <t>Cyber Security Specialist</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tata Advanced Systems Limited</t>
+          <t>BuzzClan</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Noida, Ghaziabad</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>56.25</v>
+        <v>57.27</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762127810?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=55DA7A82770C696150F83F8133FACA98264C6E3F</t>
+          <t>https://www.adzuna.in/land/ad/5753854888?se=QHteYeFu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=DCC65B6F5A7A335BD330AF1C5879E10E1A0DA2BF</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cyber Security Engineer</t>
+          <t>Cyber Security Architect</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IntraEdge</t>
+          <t>Tata Advanced Systems Limited</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Noida, Ghaziabad</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>56.12</v>
+        <v>56.25</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5754995429?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=62BBB042D860B38D9BB38703AA92E62E26E7FEEF</t>
+          <t>https://www.adzuna.in/land/ad/5762127810?se=QHteYeFu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=55DA7A82770C696150F83F8133FACA98264C6E3F</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Network Engineer</t>
+          <t>Cyber Security Engineer</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Coforge</t>
+          <t>IntraEdge</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -810,23 +810,23 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>55.7</v>
+        <v>56.12</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765773904?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=13B225115728D3657DA50775D7912A9BA4ED36EB</t>
+          <t>https://www.adzuna.in/land/ad/5754995429?se=zvWGXeFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=62BBB042D860B38D9BB38703AA92E62E26E7FEEF</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SOC Detection and Automation engineer</t>
+          <t>Cyber Security Analyst</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HCLSoftware</t>
+          <t>Landmark Group</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -835,11 +835,11 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>55.63</v>
+        <v>56.07</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765771294?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=66B0C0764A60AE7A967A48E96A0935EBE89724C7</t>
+          <t>https://www.adzuna.in/land/ad/5763491647?se=TOhCXuFu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=5573B527B75544C3C5D7FA977FB8354A34B08C75</t>
         </is>
       </c>
     </row>
@@ -851,45 +851,45 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Licious</t>
+          <t>Coforge</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>54.92</v>
+        <v>55.7</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5697518505?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=9CEC78D19FCA0C7369A7A9F85A518FE1FD101D9B</t>
+          <t>https://www.adzuna.in/land/ad/5765773904?se=hAEKX-Fu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=13B225115728D3657DA50775D7912A9BA4ED36EB</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Cyber Security Engineer</t>
+          <t>SOC Detection and Automation engineer</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Coforge</t>
+          <t>HCLSoftware</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Noida, Ghaziabad</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54.74</v>
+        <v>55.63</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753861658?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2FEC94CE5CB423BFE26CF6D30B22638EDBB7E8F1</t>
+          <t>https://www.adzuna.in/land/ad/5765771294?se=zvWGXeFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=66B0C0764A60AE7A967A48E96A0935EBE89724C7</t>
         </is>
       </c>
     </row>
@@ -901,157 +901,157 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>IH</t>
+          <t>Licious</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Thane, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54.51</v>
+        <v>54.92</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5773100081?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4E47ED62AE22E7EC84290A3E8AA04AC0672BE472</t>
+          <t>https://www.adzuna.in/land/ad/5697518505?se=hAEKX-Fu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=9CEC78D19FCA0C7369A7A9F85A518FE1FD101D9B</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Information Security Analyst</t>
+          <t>Cyber Security Engineer</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>HealthKart</t>
+          <t>Coforge</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Noida, Ghaziabad</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>54.3</v>
+        <v>54.74</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017975?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=69D84AF1829A42AB98C8A52ADFD1EFCF7612FD49</t>
+          <t>https://www.adzuna.in/land/ad/5753861658?se=QHteYeFu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2FEC94CE5CB423BFE26CF6D30B22638EDBB7E8F1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Cyber Security Analyst</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CenturyIQ</t>
+          <t>IH</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Thane, Maharashtra</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>54.06</v>
+        <v>54.51</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279314?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D58B4AE61A5DFD6033A10582B36518DC793AE0F4</t>
+          <t>https://www.adzuna.in/land/ad/5773100081?se=hAEKX-Fu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4E47ED62AE22E7EC84290A3E8AA04AC0672BE472</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Senior Network Engineer</t>
+          <t>Information Security Analyst</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>NEXPLAY SECURE</t>
+          <t>HealthKart</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>53.8</v>
+        <v>54.3</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5718579853?se=miSUf8tu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EEB22977836DEAF81366ED7E9D416316985AA188</t>
+          <t>https://www.adzuna.in/land/ad/5768017975?se=TOhCXuFu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=69D84AF1829A42AB98C8A52ADFD1EFCF7612FD49</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Network Engineer</t>
+          <t>Cyber Security Analyst</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CloudFulcrum</t>
+          <t>CenturyIQ</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>53.28</v>
+        <v>54.06</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753861185?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=764A0D94268C270F0A11F41CD71DC452D8D024EE</t>
+          <t>https://www.adzuna.in/land/ad/5769279314?se=TOhCXuFu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D58B4AE61A5DFD6033A10582B36518DC793AE0F4</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Security Analyst</t>
+          <t>Senior Network Engineer</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Searce Inc</t>
+          <t>NEXPLAY SECURE</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>52.43</v>
+        <v>53.8</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5765775462?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=37EF76F5E17E818F0447F6892E3D3033BCA9DEDB</t>
+          <t>https://www.adzuna.in/land/ad/5718579853?se=AN3UX-Fu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=EEB22977836DEAF81366ED7E9D416316985AA188</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Cyber Security Architect</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AXISCADES</t>
+          <t>CloudFulcrum</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1060,98 +1060,98 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>51.91</v>
+        <v>53.28</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747047144?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=086536F916DBD1B18D3DC8ADC94A41EDB4152A26</t>
+          <t>https://www.adzuna.in/land/ad/5753861185?se=hAEKX-Fu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=764A0D94268C270F0A11F41CD71DC452D8D024EE</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Cyber Security Specialist</t>
+          <t>Security Analyst</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ITC Infotech</t>
+          <t>Searce Inc</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>51.58</v>
+        <v>52.43</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5751935153?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=C4885E317E9A9D605051F18481BAC78ADCE69845</t>
+          <t>https://www.adzuna.in/land/ad/5765775462?se=TOhCXuFu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=37EF76F5E17E818F0447F6892E3D3033BCA9DEDB</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>System Administrator</t>
+          <t>Cyber Security Architect</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ACL Digital</t>
+          <t>AXISCADES</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>50.72</v>
+        <v>51.91</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5750488988?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D508B9EDA6796D7FEA984502C190316CE8C2A72B</t>
+          <t>https://www.adzuna.in/land/ad/5747047144?se=QHteYeFu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=086536F916DBD1B18D3DC8ADC94A41EDB4152A26</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Network Operations Center Engineer</t>
+          <t>Cyber Security Specialist</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ValueLabs</t>
+          <t>ITC Infotech</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>49.39</v>
+        <v>51.58</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753195076?se=miSUf8tu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=923801176AE7A1C9773F36AF178EBD26D512CA14</t>
+          <t>https://www.adzuna.in/land/ad/5751935153?se=QHteYeFu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=C4885E317E9A9D605051F18481BAC78ADCE69845</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Network Engineer</t>
+          <t>System Administrator</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>LTM</t>
+          <t>ACL Digital</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1160,23 +1160,23 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>49.19</v>
+        <v>50.72</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763490809?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2DE9C024149D8DBE2A1313F30D55C8D54F432F3D</t>
+          <t>https://www.adzuna.in/land/ad/5750488988?se=EpqbYOFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=D508B9EDA6796D7FEA984502C190316CE8C2A72B</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NOC Engineer (Admin)</t>
+          <t>Network Operations Center Engineer</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sonata Software</t>
+          <t>ValueLabs</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1185,123 +1185,123 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>48.24</v>
+        <v>49.39</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5742257007?se=miSUf8tu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2D757BB48A163442E841856250996D40F30FC3E4</t>
+          <t>https://www.adzuna.in/land/ad/5753195076?se=AN3UX-Fu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=923801176AE7A1C9773F36AF178EBD26D512CA14</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>System Network Administrator</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Check Point Software</t>
+          <t>LTM</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>47.56</v>
+        <v>49.19</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745164418?se=miSUf8tu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3B0A759BCDB59AF4E25E85006C1AB1D0EB157057</t>
+          <t>https://www.adzuna.in/land/ad/5763490809?se=hAEKX-Fu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2DE9C024149D8DBE2A1313F30D55C8D54F432F3D</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Network Engineer</t>
+          <t>NOC Engineer (Admin)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Persistent Systems</t>
+          <t>Sonata Software</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>47.01</v>
+        <v>48.24</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5747049084?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=125E41A1B9DDB57408262D54D83632341383D0EB</t>
+          <t>https://www.adzuna.in/land/ad/5742257007?se=AN3UX-Fu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=2D757BB48A163442E841856250996D40F30FC3E4</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Cyber Security Trainer</t>
+          <t>System Network Administrator</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PenCap Institute of Excellence</t>
+          <t>Check Point Software</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>46.24</v>
+        <v>47.56</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5760048697?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=70CA53C4D36C78E465CA1A70805E0139B2E3FFAB</t>
+          <t>https://www.adzuna.in/land/ad/5745164418?se=AN3UX-Fu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=3B0A759BCDB59AF4E25E85006C1AB1D0EB157057</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>System Administrator</t>
+          <t>Cyber Security Trainer</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Stefanini Group</t>
+          <t>PenCap Institute of Excellence</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Chennai, Tamil Nadu</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>46.19</v>
+        <v>46.24</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5757284504?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=FBC032DA8BAD5D3101B3CC9E54E5B69521B6E72A</t>
+          <t>https://www.adzuna.in/land/ad/5760048697?se=QHteYeFu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=70CA53C4D36C78E465CA1A70805E0139B2E3FFAB</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Data Security Analyst</t>
+          <t>System Administrator</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Generac</t>
+          <t>Stefanini Group</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1310,48 +1310,48 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>46.17</v>
+        <v>46.19</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5763491377?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4B3A4958BCF6866E580142C09980F0C770C32C7</t>
+          <t>https://www.adzuna.in/land/ad/5757284504?se=EpqbYOFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=FBC032DA8BAD5D3101B3CC9E54E5B69521B6E72A</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Associate Director - Cyber Security</t>
+          <t>Data Security Analyst</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Dexian India</t>
+          <t>Generac</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>44.9</v>
+        <v>46.17</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017288?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=83958946379D0B2DA69D00F6C975FEC5992724E7</t>
+          <t>https://www.adzuna.in/land/ad/5763491377?se=TOhCXuFu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4B3A4958BCF6866E580142C09980F0C770C32C7</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Network Engineer</t>
+          <t>Associate Director - Cyber Security</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Movate</t>
+          <t>Dexian India</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1360,98 +1360,98 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>44.81</v>
+        <v>44.9</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753191970?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6BDA6CC2A00FC003582875F486E3C68BB692E1A3</t>
+          <t>https://www.adzuna.in/land/ad/5768017288?se=zvWGXeFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=83958946379D0B2DA69D00F6C975FEC5992724E7</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Assistant Architect – Liaisoning (Municipal Liaisoning)</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Designo Architects</t>
+          <t>Movate</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Navi Mumbai, Maharashtra</t>
+          <t>Chennai, Tamil Nadu</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>44.2</v>
+        <v>44.81</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5750495104?se=miSUf8tu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=BEB267C4FE33B892711F37FCF4CD64F571883100</t>
+          <t>https://www.adzuna.in/land/ad/5753191970?se=hAEKX-Fu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6BDA6CC2A00FC003582875F486E3C68BB692E1A3</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>System Administrator</t>
+          <t>Assistant Architect – Liaisoning (Municipal Liaisoning)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Persistent Systems</t>
+          <t>Designo Architects</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Navi Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>43.97</v>
+        <v>44.2</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5749037378?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=439C1013C31F64FF3D99143A4ABE4BA606CE0AEF</t>
+          <t>https://www.adzuna.in/land/ad/5750495104?se=AN3UX-Fu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=BEB267C4FE33B892711F37FCF4CD64F571883100</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Senior Product Designer</t>
+          <t>System Administrator</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Unosecur</t>
+          <t>Persistent Systems</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>43.88</v>
+        <v>43.97</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5773098521?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=61A7EF41B5D62A47BAD748487EF4F5BACF71C292</t>
+          <t>https://www.adzuna.in/land/ad/5749037378?se=EpqbYOFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=439C1013C31F64FF3D99143A4ABE4BA606CE0AEF</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Data Security Analyst</t>
+          <t>Senior Product Designer</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>NuSummit Cybersecurity</t>
+          <t>Unosecur</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1460,11 +1460,11 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>43.28</v>
+        <v>43.88</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762133961?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A567A465BBFA1F3725C3B40E702992E52F05EC45</t>
+          <t>https://www.adzuna.in/land/ad/5773098521?se=zvWGXeFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=61A7EF41B5D62A47BAD748487EF4F5BACF71C292</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5374790512?se=miSUf8tu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=161F0A4DE9F0D2B630015CA623E46D4A8B0D94E6</t>
+          <t>https://www.adzuna.in/land/ad/5374790512?se=AN3UX-Fu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=161F0A4DE9F0D2B630015CA623E46D4A8B0D94E6</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5772526122?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0BA78F1159A331083EC3248C8E944199D331E6E4</t>
+          <t>https://www.adzuna.in/land/ad/5772526122?se=hAEKX-Fu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=0BA78F1159A331083EC3248C8E944199D331E6E4</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5769279202?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1DBB13C9620B1595275539972BC811719534C035</t>
+          <t>https://www.adzuna.in/land/ad/5769279202?se=EpqbYOFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1DBB13C9620B1595275539972BC811719534C035</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5677690679?se=miSUf8tu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=075C0624B177AAAB43DA3F8D6FB39E63891EAFC6</t>
+          <t>https://www.adzuna.in/land/ad/5677690679?se=AN3UX-Fu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=075C0624B177AAAB43DA3F8D6FB39E63891EAFC6</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5757286370?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F0C30441DA6E0D475D1B92065ABBB9E1AD92023</t>
+          <t>https://www.adzuna.in/land/ad/5757286370?se=TOhCXuFu8RGuCq2C_F4vAQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=8F0C30441DA6E0D475D1B92065ABBB9E1AD92023</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5721567196?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=CFA01DD69555B396E78C88671A3221E1D0E3A905</t>
+          <t>https://www.adzuna.in/land/ad/5721567196?se=EpqbYOFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=CFA01DD69555B396E78C88671A3221E1D0E3A905</t>
         </is>
       </c>
     </row>
@@ -1664,257 +1664,207 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768017103?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4F3763ADB1BAC8967835B18C3B88976D059CB89</t>
+          <t>https://www.adzuna.in/land/ad/5768017103?se=EpqbYOFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=A4F3763ADB1BAC8967835B18C3B88976D059CB89</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Information Security Analyst</t>
+          <t>Lead System Administrator</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Bahwan CyberTek</t>
+          <t>SoftTech Engineers Ltd</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>33.82</v>
+        <v>33.13</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762132173?se=LnQHfstu8RGXuJ_-STy3pQ&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=4FD2F2920AB055E5DF8BA7C040CF14891EE744D5</t>
+          <t>https://www.adzuna.in/land/ad/5762136519?se=EpqbYOFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1C916FB5C4AD09CEE16D3473EE88C0A6B6F865BB</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Lead System Administrator</t>
+          <t>NOC Engineer</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SoftTech Engineers Ltd</t>
+          <t>Harman Connected Services Corporation India Private Limited</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Pune, Maharashtra</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>33.13</v>
+        <v>32.85</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762136519?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1C916FB5C4AD09CEE16D3473EE88C0A6B6F865BB</t>
+          <t>https://www.adzuna.in/details/5716425447?utm_medium=api&amp;utm_source=df095dcc</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>NOC Engineer</t>
+          <t>Network Engineer</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Harman Connected Services Corporation India Private Limited</t>
+          <t>TekWissen India</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Pune, Maharashtra</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>32.85</v>
+        <v>29.14</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/details/5716425447?utm_medium=api&amp;utm_source=df095dcc</t>
+          <t>https://www.adzuna.in/land/ad/5762134217?se=hAEKX-Fu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=146A7355AE9AC5AC172455EB2B0E549F081EEADA</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Network Engineer</t>
+          <t>Senior System Administrator</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TekWissen India</t>
+          <t>CRS outsourcing Pvt. Ltd.</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Delhi, India</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>29.14</v>
+        <v>28.27</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5762134217?se=PpbPfstu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=146A7355AE9AC5AC172455EB2B0E549F081EEADA</t>
+          <t>https://www.adzuna.in/land/ad/5753854807?se=EpqbYOFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6142203C924F3EE1A80E3E8335EA7AF45143A5C6</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Senior System Administrator</t>
+          <t>NOC Engineer</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CRS outsourcing Pvt. Ltd.</t>
+          <t>Aeris Communications</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Delhi, India</t>
+          <t>Noida, Ghaziabad</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>28.27</v>
+        <v>28.15</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5753854807?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=6142203C924F3EE1A80E3E8335EA7AF45143A5C6</t>
+          <t>https://www.adzuna.in/details/5400411738?utm_medium=api&amp;utm_source=df095dcc</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>NOC Engineer</t>
+          <t>System Administrator</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Aeris Communications</t>
+          <t>Boutiqaat</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Noida, Ghaziabad</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>28.15</v>
+        <v>27.12</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/details/5400411738?utm_medium=api&amp;utm_source=df095dcc</t>
+          <t>https://www.adzuna.in/land/ad/5768018385?se=EpqbYOFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1BF74BBEF1DAFDEE41395186E5489C69F4BEE8BC</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>System Administrator</t>
+          <t>EVP Cyber Security</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Boutiqaat</t>
+          <t>VISTRA</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>27.12</v>
+        <v>20.18</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5768018385?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=1BF74BBEF1DAFDEE41395186E5489C69F4BEE8BC</t>
+          <t>https://www.adzuna.in/land/ad/5745167451?se=QHteYeFu8RG3pc9h1tgKVA&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1B7A588380034AAC42D886A7592B02CBF24E34A</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>EVP Cyber Security</t>
+          <t>Systems Administrator</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>VISTRA</t>
+          <t>Lexitas</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Mumbai, Maharashtra</t>
+          <t>Chennai, Tamil Nadu</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>20.18</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5745167451?se=MFkngctu8RGOUJ6zGKp4Eg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1B7A588380034AAC42D886A7592B02CBF24E34A</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Cyber Incident Response Lead</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Owens &amp; Minor</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="D59" t="n">
-        <v>11.92</v>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.in/land/ad/5745166822?se=FPlMfctu8RGQCdTqtj6PDg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=75DC13623E0BEA957F10FDAE9EDE19728AAF88FE</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Systems Administrator</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Lexitas</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Chennai, Tamil Nadu</t>
-        </is>
-      </c>
-      <c r="D60" t="n">
-        <v>9.619999999999999</v>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.in/land/ad/5737585201?se=EkJigMtu8RGU18viNYDoqg&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1E457E6EF8E102A87845B46934F33F96B5E3422</t>
+          <t>https://www.adzuna.in/land/ad/5737585201?se=EpqbYOFu8RGyv4cQeQGO3g&amp;utm_medium=api&amp;utm_source=df095dcc&amp;v=B1E457E6EF8E102A87845B46934F33F96B5E3422</t>
         </is>
       </c>
     </row>

</xml_diff>